<commit_message>
Add Use case Description
</commit_message>
<xml_diff>
--- a/hw1/Use_case_descriptions/Use_case_descriptions.xlsx
+++ b/hw1/Use_case_descriptions/Use_case_descriptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscar/Desktop/4th_grade/1st/Software_Engineering/hw/hw1/Use_case_descriptions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85600850-4649-364F-A743-705A88DA559D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666315B1-0360-8848-A6FE-12D8969C8E33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{2F6E1894-1E13-4ED7-A12D-A34235E4ED08}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{2F6E1894-1E13-4ED7-A12D-A34235E4ED08}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>No.</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -151,6 +151,42 @@
   </si>
   <si>
     <t>5.조건에 맞는 설문리스트 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. ID, 비밀번호, 이름, 전화번호, 이메일 입력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. 회원 탈퇴 버튼 클릭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. ID, 비밀번호 입력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. 로그인 완료 화면 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. 탈퇴 완료 창 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 로그인 화면 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 회원 탈퇴 화면 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. 계정 생성 완료 창 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 회원 가입 화면 출력</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -158,7 +194,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,6 +210,14 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -183,7 +227,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -195,24 +239,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -226,13 +252,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -244,24 +263,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -271,13 +272,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -287,35 +301,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -651,196 +674,343 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFAF8D5E-662B-45C9-986E-8317241416BC}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="54.1640625" customWidth="1"/>
+    <col min="2" max="2" width="59.5" customWidth="1"/>
     <col min="3" max="3" width="38.5" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="52.1640625" customWidth="1"/>
+    <col min="7" max="7" width="35.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="19.5" customHeight="1">
+    <row r="1" spans="1:11" ht="19.5" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="E2" s="15"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" s="6">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="6">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="7"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="10">
         <v>4</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="6"/>
-      <c r="B4" t="s">
+    <row r="13" spans="1:11">
+      <c r="A13" s="10"/>
+      <c r="B13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="7"/>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="6"/>
-      <c r="C5" s="7" t="s">
+      <c r="C13" s="7"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="10"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="6"/>
-      <c r="B6" t="s">
+    <row r="15" spans="1:11">
+      <c r="A15" s="10"/>
+      <c r="B15" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="7"/>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="6"/>
-      <c r="C7" s="7" t="s">
+      <c r="C15" s="7"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="10"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="8" t="s">
+    <row r="17" spans="1:3">
+      <c r="A17" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="6"/>
-      <c r="B9" t="s">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="10"/>
+      <c r="B18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="6"/>
-      <c r="C10" s="7" t="s">
+      <c r="C18" s="7"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="10"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="6"/>
-      <c r="B11" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" s="10"/>
+      <c r="B20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="7"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="6"/>
-      <c r="C12" s="7" t="s">
+      <c r="C20" s="7"/>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="10"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="6"/>
-      <c r="B13" t="s">
+    <row r="22" spans="1:3">
+      <c r="A22" s="10"/>
+      <c r="B22" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="7"/>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="6"/>
-      <c r="C14" s="7" t="s">
+      <c r="C22" s="7"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="6"/>
-      <c r="B15" t="s">
+    <row r="24" spans="1:3">
+      <c r="A24" s="10"/>
+      <c r="B24" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="7"/>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11" t="s">
+      <c r="C24" s="7"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="11"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="6">
+    <row r="26" spans="1:3">
+      <c r="A26" s="10">
         <v>5</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="B26" s="7"/>
+      <c r="C26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="6"/>
-      <c r="B18" t="s">
+    <row r="27" spans="1:3">
+      <c r="A27" s="10"/>
+      <c r="B27" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="7"/>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="6"/>
-      <c r="C19" s="7" t="s">
+      <c r="C27" s="7"/>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="10"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="8" t="s">
+    <row r="29" spans="1:3">
+      <c r="A29" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="7"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="6"/>
-      <c r="B21" t="s">
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="10"/>
+      <c r="B30" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="7"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="6"/>
-      <c r="C22" s="7" t="s">
+      <c r="C30" s="7"/>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="11"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="3">
+    <row r="32" spans="1:3">
+      <c r="A32" s="5">
         <v>6</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="5" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="36">
-      <c r="A24" s="6"/>
-      <c r="B24" s="12" t="s">
+    <row r="33" spans="1:3" ht="36">
+      <c r="A33" s="10"/>
+      <c r="B33" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="7"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="6"/>
-      <c r="C25" s="7" t="s">
+      <c r="C33" s="7"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="10"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="6"/>
-      <c r="B26" t="s">
+    <row r="35" spans="1:3">
+      <c r="A35" s="10"/>
+      <c r="B35" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="7"/>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="9"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11" t="s">
+      <c r="C35" s="7"/>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="11"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>